<commit_message>
formata xlsx (larguras, cabecalho, filtro, freeze)
</commit_message>
<xml_diff>
--- a/data/processed/resultado.xlsx
+++ b/data/processed/resultado.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="resultado" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'resultado'!$A$1:$J$108</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -29,12 +31,18 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -55,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,54 +438,66 @@
   </sheetPr>
   <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>consulta_logradouro</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>consulta_numero</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>consulta_bairro</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>consulta_cep</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>consulta_complemento</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>consulta_municipio</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>setor_censitario_encontrado</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>match_status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>match_layer</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>match_score</t>
         </is>
@@ -486,7 +509,6 @@
           <t>RODOVIA BR 101</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>BR101</t>
@@ -545,7 +567,6 @@
           <t>46830000</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>290130</t>
@@ -574,8 +595,6 @@
           <t>FAZENDA BICO</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>46130000</t>
@@ -629,7 +648,6 @@
           <t>45675000</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>290240</t>
@@ -673,7 +691,6 @@
           <t>47800020</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>290320</t>
@@ -717,7 +734,6 @@
           <t>45860000</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>290630</t>
@@ -746,8 +762,6 @@
           <t>FAZENDA LAGOA GRANDE</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>46380000</t>
@@ -839,13 +853,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>48110000</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>290750</t>
@@ -879,13 +891,11 @@
           <t>89</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>45822000</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>291072</t>
@@ -929,7 +939,6 @@
           <t>44010231</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>291080</t>
@@ -963,7 +972,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>44350000</t>
@@ -1017,7 +1025,6 @@
           <t>46430000</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>291170</t>
@@ -1099,13 +1106,11 @@
           <t>23</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>45745000</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>291210</t>
@@ -1245,7 +1250,6 @@
           <t>45607000</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>291480</t>
@@ -1289,7 +1293,6 @@
           <t>45836000</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>291560</t>
@@ -1371,13 +1374,11 @@
           <t>389</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>45780000</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>291680</t>
@@ -1421,7 +1422,6 @@
           <t>48960000</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>291770</t>
@@ -1455,13 +1455,11 @@
           <t>23</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>48905000</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>291840</t>
@@ -1505,7 +1503,6 @@
           <t>45490000</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>291880</t>
@@ -1549,7 +1546,6 @@
           <t>45490000</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>291880</t>
@@ -1593,7 +1589,6 @@
           <t>48720000</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>291910</t>
@@ -1685,7 +1680,6 @@
           <t>45255000</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>292145</t>
@@ -1729,7 +1723,6 @@
           <t>45890000</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>292390</t>
@@ -1773,7 +1766,6 @@
           <t>47240000</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>292440</t>
@@ -1807,13 +1799,11 @@
           <t>237</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>48120000</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>292520</t>
@@ -1857,7 +1847,6 @@
           <t>45810000</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>292530</t>
@@ -1891,13 +1880,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>45816000</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>292530</t>
@@ -1931,13 +1918,11 @@
           <t>508</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>45810000</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>292530</t>
@@ -1981,7 +1966,6 @@
           <t>45810000</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>292530</t>
@@ -2025,7 +2009,6 @@
           <t>48860000</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>292580</t>
@@ -2117,7 +2100,6 @@
           <t>40750670</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>292740</t>
@@ -2161,7 +2143,6 @@
           <t>41190000</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>292740</t>
@@ -2205,7 +2186,6 @@
           <t>41925540</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>292740</t>
@@ -2249,7 +2229,6 @@
           <t>41290001</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>292740</t>
@@ -2283,13 +2262,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>40470380</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>292740</t>
@@ -2323,13 +2300,11 @@
           <t>49</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>40370330</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>292740</t>
@@ -2363,7 +2338,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>40820060</t>
@@ -2417,7 +2391,6 @@
           <t>44190000</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>292880</t>
@@ -2446,8 +2419,6 @@
           <t>SITIO ESPERANCA</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>48895000</t>
@@ -2501,7 +2472,6 @@
           <t>48700000</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>293050</t>
@@ -2545,7 +2515,6 @@
           <t>48925000</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>293077</t>
@@ -2589,7 +2558,6 @@
           <t>45998000</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>293135</t>
@@ -2618,7 +2586,6 @@
           <t>FAZENDA QUEIMADA DOS PADEIROS</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>QUEIMADAS DOS LOIOLAS</t>
@@ -2677,7 +2644,6 @@
           <t>45545000</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>293220</t>
@@ -2721,7 +2687,6 @@
           <t>45690000</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>293250</t>
@@ -2765,7 +2730,6 @@
           <t>44470000</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>293320</t>
@@ -2809,7 +2773,6 @@
           <t>47400000</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>293360</t>
@@ -2838,8 +2801,6 @@
           <t>AVENIDA CALDEIRO DA VACA</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>48990000</t>
@@ -2893,7 +2854,6 @@
           <t>44620000</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>290260</t>
@@ -2937,7 +2897,6 @@
           <t>47800200</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>290320</t>
@@ -3029,7 +2988,6 @@
           <t>45800000</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>290340</t>
@@ -3063,13 +3021,11 @@
           <t>68</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>47600000</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>290390</t>
@@ -3098,7 +3054,6 @@
           <t>RUA AMAZONAS</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>MALEMBA DE BAIXO</t>
@@ -3243,7 +3198,6 @@
           <t>18</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>44500000</t>
@@ -3287,13 +3241,11 @@
           <t>42</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>48730000</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>290840</t>
@@ -3375,13 +3327,11 @@
           <t>315</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>48480000</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>290960</t>
@@ -3463,13 +3413,11 @@
           <t>147</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>45840000</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>291180</t>
@@ -3498,8 +3446,6 @@
           <t>RUA SANTA ISABEL</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>46860000</t>
@@ -3553,7 +3499,6 @@
           <t>45570000</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>291390</t>
@@ -3597,7 +3542,6 @@
           <t>44900000</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>291460</t>
@@ -3641,7 +3585,6 @@
           <t>45607000</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>291480</t>
@@ -3675,13 +3618,11 @@
           <t>103</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>45455000</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>291570</t>
@@ -3725,7 +3666,6 @@
           <t>44460000</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>291610</t>
@@ -3759,13 +3699,11 @@
           <t>57</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
           <t>45350000</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>291690</t>
@@ -3809,7 +3747,6 @@
           <t>44700000</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>291750</t>
@@ -3853,7 +3790,6 @@
           <t>45206000</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>291800</t>
@@ -3887,7 +3823,6 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>48905000</t>
@@ -3926,8 +3861,6 @@
           <t>RUA JULIO VERNE</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>47850000</t>
@@ -3971,13 +3904,11 @@
           <t>250</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
           <t>44575000</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>292220</t>
@@ -4069,7 +4000,6 @@
           <t>48870000</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>292265</t>
@@ -4242,8 +4172,6 @@
           <t>RUA ADEGUNDES ARAUJO</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>45890000</t>
@@ -4287,13 +4215,11 @@
           <t>41</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>44830000</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>292480</t>
@@ -4337,7 +4263,6 @@
           <t>45190000</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>292500</t>
@@ -4462,8 +4387,6 @@
           <t>AVENIDA LEOVIGILDO FILGUEIRAS</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>40421020</t>
@@ -4565,7 +4488,6 @@
           <t>41400000</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>292740</t>
@@ -4599,7 +4521,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>41340295</t>
@@ -4691,7 +4612,6 @@
           <t>26</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>40735560</t>
@@ -4735,7 +4655,6 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>41611685</t>
@@ -4827,13 +4746,11 @@
           <t>33</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
           <t>44571050</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>292870</t>
@@ -4877,7 +4794,6 @@
           <t>44190000</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>292880</t>
@@ -4921,7 +4837,6 @@
           <t>44550000</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>292910</t>
@@ -4965,7 +4880,6 @@
           <t>44915000</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>292925</t>
@@ -5009,7 +4923,6 @@
           <t>43850000</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>292950</t>
@@ -5091,13 +5004,11 @@
           <t>169</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>47630000</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>293015</t>
@@ -5141,7 +5052,6 @@
           <t>44270000</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>293170</t>
@@ -5165,6 +5075,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>